<commit_message>
Backfill: tracked horses through 2026-06-11
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,279 @@
         <v>46246</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Backfill: tracked horses through 2026-07-11
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,15 +519,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>York</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46277</v>
+        <v>46254</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46170</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46170</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,11 +675,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,11 +714,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -777,6 +777,162 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
         <v>46170</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>James J Braddock</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" s="1" t="n">
+        <v>46184</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Port Ferdinand</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" s="1" t="n">
+        <v>46196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill: tracked horses through 2026-08-10
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +722,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46170</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="9">
@@ -800,7 +800,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46184</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="11">
@@ -839,7 +839,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46170</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="12">
@@ -878,7 +878,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46170</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="13">
@@ -933,6 +933,318 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
         <v>46196</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" s="1" t="n">
+        <v>46238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill: tracked horses complete through 2026-08-15
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,46 +470,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The Institute</t>
+          <t>Equus Victor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FINGER LAKES</t>
+          <t>Dundalk</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>final entry</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>virtualstable</t>
+          <t>horsetracker</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,20 +519,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Deauville</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46254</v>
+        <v>46249</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,13 +542,13 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46210</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Sir Alfie</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,20 +558,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Lingfield</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46277</v>
+        <v>46249</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46170</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Wimbledon Hawkeye</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,20 +597,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Deauville</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46277</v>
+        <v>46249</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,36 +620,36 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46184</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Without Compromise</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Pontefract</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46277</v>
+        <v>46250</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -659,13 +659,13 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46170</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Bucaneer's Spirit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,15 +675,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46277</v>
+        <v>46252</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -698,52 +698,52 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46170</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>The Institute</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>FINGER LAKES</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46277</v>
+        <v>46252</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>final entry</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>horsetracker</t>
+          <t>virtualstable</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46232</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -753,15 +753,15 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Carlisle</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46278</v>
+        <v>46253</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -776,31 +776,31 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46170</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>York</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46278</v>
+        <v>46253</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46232</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,15 +831,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>York</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46278</v>
+        <v>46254</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -854,13 +854,13 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46232</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -870,15 +870,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -893,27 +893,27 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46232</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Port Ferdinand</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -932,13 +932,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46196</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -948,15 +948,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46298</v>
+        <v>46277</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -971,13 +971,13 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -987,15 +987,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1010,31 +1010,31 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1049,13 +1049,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1065,15 +1065,15 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1088,31 +1088,31 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1127,13 +1127,13 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1143,15 +1143,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1166,31 +1166,31 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1205,31 +1205,31 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Port Ferdinand</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1244,6 +1244,318 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-08-16
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Equus Victor</t>
+          <t>A Boy Named Susie</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dundalk</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,13 +503,13 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Alrashdeyah</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,20 +519,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Deauville</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -548,7 +548,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sir Alfie</t>
+          <t>Angels Have Wings</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,20 +558,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lingfield</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,36 +581,36 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Away And Gone</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Deauville</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -626,17 +626,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Without Compromise</t>
+          <t>Coincidenza</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pontefract</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -644,12 +644,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bucaneer's Spirit</t>
+          <t>Cowardofthecounty</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,20 +675,20 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Roscommon</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46252</v>
+        <v>46250</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -698,75 +698,75 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The Institute</t>
+          <t>Dancinginthecity</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FINGER LAKES</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46252</v>
+        <v>46250</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>final entry</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>virtualstable</t>
+          <t>horsetracker</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46246</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Count Palatine</t>
+          <t>Moon Sand</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Carlisle</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46253</v>
+        <v>46250</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,13 +776,13 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Mr Montauk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -792,20 +792,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46253</v>
+        <v>46250</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Omni Man</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,20 +831,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46254</v>
+        <v>46250</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -860,7 +860,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Star Prospect</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -870,20 +870,20 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46277</v>
+        <v>46250</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -893,36 +893,36 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46170</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Tommy Quick</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46277</v>
+        <v>46250</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -932,36 +932,36 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46184</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Without Compromise</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Pontefract</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46277</v>
+        <v>46250</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -971,13 +971,13 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46170</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Zarak Pasha</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -987,20 +987,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46277</v>
+        <v>46250</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1010,13 +1010,13 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46170</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Bucaneer's Spirit</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1026,15 +1026,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46277</v>
+        <v>46252</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1049,70 +1049,70 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46232</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>The Institute</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>FINGER LAKES</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46278</v>
+        <v>46252</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>final entry</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>horsetracker</t>
+          <t>virtualstable</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46170</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Carlisle</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46278</v>
+        <v>46253</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1127,13 +1127,13 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46232</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1143,15 +1143,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>York</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46278</v>
+        <v>46253</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1166,13 +1166,13 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46232</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1182,15 +1182,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>York</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46278</v>
+        <v>46254</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1205,13 +1205,13 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46232</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Port Ferdinand</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1221,11 +1221,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1244,31 +1244,31 @@
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" s="1" t="n">
-        <v>46196</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>46298</v>
+        <v>46277</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1283,13 +1283,13 @@
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" s="1" t="n">
-        <v>46238</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1299,15 +1299,15 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1322,31 +1322,31 @@
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1361,13 +1361,13 @@
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1377,15 +1377,15 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1400,13 +1400,13 @@
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1416,15 +1416,15 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1439,31 +1439,31 @@
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" s="1" t="n">
-        <v>46238</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1478,31 +1478,31 @@
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D28" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1517,31 +1517,31 @@
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" s="1" t="n">
-        <v>46238</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Curragh</t>
         </is>
       </c>
       <c r="D29" s="1" t="n">
-        <v>46312</v>
+        <v>46278</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1556,6 +1556,357 @@
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" s="1" t="n">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Port Ferdinand</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-08-23
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A Boy Named Susie</t>
+          <t>Equus Victor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Navan</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46250</v>
+        <v>46261</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,13 +503,13 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46248</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alrashdeyah</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,20 +519,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46250</v>
+        <v>46277</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,36 +542,36 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46248</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Angels Have Wings</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46250</v>
+        <v>46277</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46248</v>
+        <v>46184</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Away And Gone</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,20 +597,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46250</v>
+        <v>46277</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46248</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Coincidenza</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -636,20 +636,20 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46250</v>
+        <v>46277</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -659,13 +659,13 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46248</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cowardofthecounty</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,20 +675,20 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Leopardstown</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46250</v>
+        <v>46277</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -698,13 +698,13 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46248</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dancinginthecity</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -718,16 +718,16 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46250</v>
+        <v>46278</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -737,18 +737,18 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46248</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moon Sand</t>
+          <t>James J Braddock</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -757,16 +757,16 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46250</v>
+        <v>46278</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,13 +776,13 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46248</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mr Montauk</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -796,16 +796,16 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46250</v>
+        <v>46278</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13:35</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -815,13 +815,13 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46248</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Omni Man</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -835,16 +835,16 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46250</v>
+        <v>46278</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -854,13 +854,13 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46248</v>
+        <v>46232</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Star Prospect</t>
+          <t>Port Ferdinand</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46250</v>
+        <v>46278</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -893,36 +893,36 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46248</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tommy Quick</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Newmarket</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46250</v>
+        <v>46298</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -932,36 +932,36 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46248</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Without Compromise</t>
+          <t>Benvenuto Cellini</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pontefract</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46250</v>
+        <v>46312</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>declared</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -971,36 +971,36 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46248</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zarak Pasha</t>
+          <t>Erdenali</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46250</v>
+        <v>46312</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>runs</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1010,13 +1010,13 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46248</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bucaneer's Spirit</t>
+          <t>Pierre Bonnard</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1026,15 +1026,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Roscommon</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46252</v>
+        <v>46312</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1049,52 +1049,52 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46247</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>The Institute</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FINGER LAKES</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46252</v>
+        <v>46312</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>final entry</t>
+          <t>entered</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>virtualstable</t>
+          <t>horsetracker</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46246</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Count Palatine</t>
+          <t>Sparan Nua</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1104,15 +1104,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Carlisle</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46253</v>
+        <v>46312</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1127,31 +1127,31 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46247</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>White Birch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46253</v>
+        <v>46312</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1166,31 +1166,31 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46247</v>
+        <v>46238</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Wimbledon Hawkeye</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Ascot</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46254</v>
+        <v>46312</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1205,708 +1205,6 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Benvenuto Cellini</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Leopardstown</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" s="1" t="n">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>James J Braddock</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Leopardstown</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" s="1" t="n">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Montreal</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Leopardstown</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" s="1" t="n">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Pierre Bonnard</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Leopardstown</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" s="1" t="n">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Puerto Rico</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Leopardstown</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" s="1" t="n">
-        <v>46232</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Benvenuto Cellini</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Curragh</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" s="1" t="n">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>James J Braddock</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Curragh</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>16:35</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" s="1" t="n">
-        <v>46232</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Montreal</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Curragh</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>16:35</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" s="1" t="n">
-        <v>46232</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Pierre Bonnard</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Curragh</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>16:35</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" s="1" t="n">
-        <v>46232</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Port Ferdinand</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Curragh</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" s="1" t="n">
-        <v>46196</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Sparan Nua</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Newmarket</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>46298</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Benvenuto Cellini</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Erdenali</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>14:40</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Pierre Bonnard</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Puerto Rico</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>14:40</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Sparan Nua</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>IRE</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>14:05</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>White Birch</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D37" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" s="1" t="n">
-        <v>46238</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wimbledon Hawkeye</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Ascot</t>
-        </is>
-      </c>
-      <c r="D38" s="1" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>entered</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>horsetracker</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly tracked-horses update through 2026-08-30
</commit_message>
<xml_diff>
--- a/data/tracked/tracked-horses.xlsx
+++ b/data/tracked/tracked-horses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Equus Victor</t>
+          <t>Aiteall</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,20 +480,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Navan</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46261</v>
+        <v>46264</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,13 +503,13 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="1" t="n">
-        <v>46254</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Count Palatine</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,20 +519,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Beverley</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46277</v>
+        <v>46264</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -542,36 +542,36 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="1" t="n">
-        <v>46170</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Dancing Saxon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>46277</v>
+        <v>46264</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -581,13 +581,13 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" s="1" t="n">
-        <v>46184</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Dang Thai Son</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -597,20 +597,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46277</v>
+        <v>46264</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,13 +620,13 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" s="1" t="n">
-        <v>46170</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Eighteenth Smiles</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -636,20 +636,20 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>46277</v>
+        <v>46264</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -659,13 +659,13 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" s="1" t="n">
-        <v>46170</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Feel Happy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,20 +675,20 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Leopardstown</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46277</v>
+        <v>46264</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -698,13 +698,13 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" s="1" t="n">
-        <v>46232</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Felix Guido</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,20 +714,20 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46278</v>
+        <v>46264</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -737,36 +737,36 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" s="1" t="n">
-        <v>46170</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>James J Braddock</t>
+          <t>Greydreambeliever</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46278</v>
+        <v>46264</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,13 +776,13 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" s="1" t="n">
-        <v>46232</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Josh's Joy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -792,20 +792,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46278</v>
+        <v>46264</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -815,36 +815,36 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" s="1" t="n">
-        <v>46232</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Princess Child</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46278</v>
+        <v>46264</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -854,13 +854,13 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" s="1" t="n">
-        <v>46232</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Port Ferdinand</t>
+          <t>Spinning Around</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -870,20 +870,20 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Curragh</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46278</v>
+        <v>46264</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -893,36 +893,36 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" s="1" t="n">
-        <v>46196</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Stugardia</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IRE</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Newmarket</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46298</v>
+        <v>46264</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -932,13 +932,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" s="1" t="n">
-        <v>46238</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Benvenuto Cellini</t>
+          <t>Togetherwearefree</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -948,20 +948,20 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Cork</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46312</v>
+        <v>46264</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -971,36 +971,36 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" s="1" t="n">
-        <v>46238</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Erdenali</t>
+          <t>Augusta Rock</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1010,13 +1010,13 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" s="1" t="n">
-        <v>46238</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pierre Bonnard</t>
+          <t>Dial Me In</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1026,20 +1026,20 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1049,13 +1049,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" s="1" t="n">
-        <v>46238</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Divilabother</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Cartmel</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>declared</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1088,13 +1088,13 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" s="1" t="n">
-        <v>46238</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sparan Nua</t>
+          <t>Equus Victor</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1104,15 +1104,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1127,36 +1127,36 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" s="1" t="n">
-        <v>46238</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>White Birch</t>
+          <t>Fratas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IRE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1166,36 +1166,36 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" s="1" t="n">
-        <v>46238</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Wimbledon Hawkeye</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>GER</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ascot</t>
+          <t>Roscommon</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46312</v>
+        <v>46265</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>entered</t>
+          <t>runs</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,6 +1205,1137 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Imperial Merlin</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cartmel</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>declared</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mawhibah</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Metallic</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ruler's Control</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sinmara</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>runs</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>The Institute</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>FINGER LAKES</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>16:18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>final entry</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>virtualstable</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" s="1" t="n">
+        <v>46259</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Equus Victor</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Gowran Park</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" s="1" t="n">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fortitudine</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Kempton</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" s="1" t="n">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sir Alfie</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Lingfield</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" s="1" t="n">
+        <v>46262</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Divilabother</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Bangor-on-Dee</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" s="1" t="n">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>James J Braddock</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" s="1" t="n">
+        <v>46184</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Leopardstown</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" s="1" t="n">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" s="1" t="n">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>James J Braddock</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" s="1" t="n">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" s="1" t="n">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" s="1" t="n">
+        <v>46232</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Port Ferdinand</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Curragh</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Snellen</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Gowran Park</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" s="1" t="n">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Newmarket</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Benvenuto Cellini</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Erdenali</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Pierre Bonnard</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sparan Nua</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>IRE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>White Birch</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" s="1" t="n">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Wimbledon Hawkeye</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Ascot</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>entered</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>horsetracker</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" s="1" t="n">
         <v>46238</v>
       </c>
     </row>

</xml_diff>